<commit_message>
Hardware: apply the lead's answers DQ-011, -049, -051, -063, -064, -065, -114
- DQ-063: WP-H-04 keeps SG-01 at ASIL C targets with the ASIL B result
  alongside; OI-2 closed.
- DQ-065: route to schematic and BOM is ask comma.ai and wait, no
  teardown (WP-H-02 OI-1, WP-H-01 OI-3, WP-H-04/05 plans, WP-H-07 OI-5).
- DQ-051: added hardware allowed in principle from the metric results
  within a budget (WP-H-01 OI-6, WP-H-04 plan step 7).
- DQ-011: both boards stay in scope (WP-H-01 OI-7, WP-H-02 OI-3, WP-H-04,
  DFMEA diagram data).
- DQ-049: HIL bench deferred; WP-H-06 T-HIL/FI cases blocked, OI-1;
  WP-H-04 plan step 5; DFM-ACT-003.
- DQ-064: WP-H-03 OI-9 closed: warn and refuse to engage.
- DQ-114: IWDG DC credit in FMEDA SG-009 provisional until the
  independent review and LSI tolerance check (WP-H-04 status note).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xx6vAdwvGpomGg8X6smJDx
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/dfmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/dfmea-review.xlsx
@@ -2445,7 +2445,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Run the watchdog HIL test (test_10_hw_watchdog) on the bench and confirm the relay releases on reset (HWSR-502, UK-06) (D-04)</t>
+            <t>Run the watchdog HIL test (test_10_hw_watchdog) on the bench and confirm the relay releases on reset (HWSR-502, UK-06) (D-04). The lead deferred the HIL bench (DQ-049, 2026-10-14), so this waits for the bench</t>
           </r>
         </is>
       </c>
@@ -2991,7 +2991,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Run the watchdog HIL test (test_10_hw_watchdog) on the bench and confirm the relay releases on reset (HWSR-502, UK-06) (D-04)</t>
+            <t>Run the watchdog HIL test (test_10_hw_watchdog) on the bench and confirm the relay releases on reset (HWSR-502, UK-06) (D-04). The lead deferred the HIL bench (DQ-049, 2026-10-14), so this waits for the bench</t>
           </r>
         </is>
       </c>
@@ -8181,7 +8181,7 @@
       <c r="H3" s="53" t="inlineStr"/>
       <c r="I3" s="53" t="inlineStr"/>
     </row>
-    <row r="4" ht="33" customHeight="1">
+    <row r="4" ht="60" customHeight="1">
       <c r="A4" s="53" t="inlineStr">
         <is>
           <t>DFM-ACT-003</t>
@@ -8194,7 +8194,7 @@
       </c>
       <c r="C4" s="53" t="inlineStr">
         <is>
-          <t>Run the watchdog HIL test (test_10_hw_watchdog) on the bench and confirm the relay releases on reset (HWSR-502, UK-06) (D-04)</t>
+          <t>Run the watchdog HIL test (test_10_hw_watchdog) on the bench and confirm the relay releases on reset (HWSR-502, UK-06) (D-04). The lead deferred the HIL bench (DQ-049, 2026-10-14), so this waits for the bench</t>
         </is>
       </c>
       <c r="D4" s="53" t="inlineStr">

</xml_diff>

<commit_message>
DFMEA rev 0.7: move to baseline BL-005
The hardware is unchanged. The panda changes 9f60e17..a55bdfc that touch
DFMEA rows were read at the pins: 0.3 s heartbeat revocation, watchdog
reset in health, IRQ priorities, reference-build flag, siren on
heartbeat loss and persistent EPS fault, ELM327 gate. The reference
build is the default at BL-005.

- S, O, D and AP unchanged.
- MSR: DFM-009.C1 M 8 -> 6 (host controlsMismatch within 0.5 s, TSR-621,
  puts the warning at about 0.66 s, inside 1 s).
- DFM-017: panda siren listed as mechanism; C1/C2 enter MSR scope at
  M 10 (nothing checks the speaker path without the SoC).
- DFM-004, DFM-015, DFM-016 text updated for BL-005 and the box pull-down.
- msr-plan §4.7 DFMEA at BL-005 table; fmea-plan DFMEA line.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xx6vAdwvGpomGg8X6smJDx
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/dfmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/dfmea-review.xlsx
@@ -781,7 +781,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.6 · draft</t>
+          <t>0.7 · draft</t>
         </is>
       </c>
     </row>
@@ -793,7 +793,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>BL-002</t>
+          <t>BL-005</t>
         </is>
       </c>
     </row>
@@ -829,7 +829,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Safety-relevant hardware of AC-001 at BL-002: comma 3X panda section (STM32H725, clock and watchdog, MCU supply, CAN transceivers), Toyota harness and relay box, SoC-MCU interface, siren path, enclosure and cooling. SoC, cameras and other QM hardware only where they couple into these (WP-A-03).</t>
+          <t>Safety-relevant hardware of AC-001 at BL-005 (hardware as at BL-002): comma 3X panda section (STM32H725, clock and watchdog, MCU supply, CAN transceivers), Toyota harness and relay box, SoC-MCU interface, siren path, enclosure and cooling. SoC, cameras and other QM hardware only where they couple into these (WP-A-03).</t>
         </is>
       </c>
     </row>
@@ -5713,7 +5713,7 @@
       <c r="R22" s="39" t="inlineStr"/>
       <c r="S22" s="39" t="inlineStr"/>
     </row>
-    <row r="23" ht="154.5" customHeight="1">
+    <row r="23" ht="168" customHeight="1">
       <c r="A23" s="30" t="inlineStr">
         <is>
           <r>
@@ -5913,7 +5913,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>• 8-bit XOR on header and data, NACK on mismatch (drivers/spi.h:97-138); reference lock limits what a corrupted 0xdc can select (reference build only)</t>
+            <t>• 8-bit XOR on header and data, NACK on mismatch (drivers/spi.h:97-138); reference lock limits what a corrupted 0xdc can select (default build from BL-005, LionDriver</t>
           </r>
           <r>
             <rPr>
@@ -8033,7 +8033,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LDFMEA — device, integrated panda, harness, vehicle interfaces · rev 0.6 · BL-002&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LDFMEA — device, integrated panda, harness, vehicle interfaces · rev 0.7 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
FMEA-MSR M3: MSR sheet in the System FMEA and DFMEA review workbooks
fmea_review_xlsx.py adds a sheet "MSR" where the analysis has FMEA-MSR
rows: one row per in-scope cause with diagnostic, system response, effect
after the response, S after, F, M, MSR AP (colour-coded), timing against
the FTTI, basis, monitoring actions with status, and the reviewer
columns; exempt causes show their reason. The cover adds MSR AP and
monitoring-band counts, and both say the MSR AP table is provisional.
The AIAG-VDA worksheet column order is unchanged. Tests for the row set,
MSR AP against fmea_lint and the absence of the sheet without MSR rows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/dfmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/dfmea-review.xlsx
@@ -11,12 +11,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worksheet" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actions" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structure" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MSR" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$30</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Worksheet'!$1:$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Structure'!$A$1:$E$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'MSR'!$A$2:$P$21</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'MSR'!$1:$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -252,7 +255,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -378,6 +381,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -744,7 +750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:C33"/>
+  <dimension ref="B2:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -914,104 +920,112 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>FMEA-MSR (msr: complete)</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>19 rated, 0 exempt; MSR AP H 19, M 0, L 0 (provisional table)</t>
+        </is>
+      </c>
+    </row>
     <row r="21">
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Monitoring M</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>1–4: 0 · 5–6: 0 · 7–8: 5 · 9–10: 14 (see sheet MSR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>Legend</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="12" t="inlineStr">
+    <row r="24">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="C22" s="13" t="inlineStr">
+      <c r="C24" s="13" t="inlineStr">
         <is>
           <t>High: an action or a rationale is required</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" s="14" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="14" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C23" s="13" t="inlineStr">
+      <c r="C25" s="13" t="inlineStr">
         <is>
           <t>Medium: an action or a rationale is recommended</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="15" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="15" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="C24" s="13" t="inlineStr">
+      <c r="C26" s="13" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="16" t="inlineStr">
+    <row r="27">
+      <c r="B27" s="16" t="inlineStr">
         <is>
           <t>Aa</t>
         </is>
       </c>
-      <c r="C25" s="13" t="inlineStr">
+      <c r="C27" s="13" t="inlineStr">
         <is>
           <t>Amber text: no test targets the cause (detection 9 or 10)</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="17" t="inlineStr"/>
-      <c r="C26" s="13" t="inlineStr">
+    <row r="28">
+      <c r="B28" s="17" t="inlineStr"/>
+      <c r="C28" s="13" t="inlineStr">
         <is>
           <t>Yellow cells on the Worksheet: reviewer input (decision from the list, comment)</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="6" t="inlineStr">
+    <row r="30">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>Review sign-off</t>
         </is>
       </c>
-    </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="B29" s="18" t="inlineStr">
-        <is>
-          <t>Reviewer</t>
-        </is>
-      </c>
-      <c r="C29" s="19" t="inlineStr"/>
-    </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="B30" s="18" t="inlineStr">
-        <is>
-          <t>Independence level</t>
-        </is>
-      </c>
-      <c r="C30" s="19" t="inlineStr"/>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Reviewer</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr"/>
     </row>
-    <row r="32" ht="30" customHeight="1">
+    <row r="32" ht="18" customHeight="1">
       <c r="B32" s="18" t="inlineStr">
         <is>
-          <t>Result (accepted / accepted with findings / rejected)</t>
+          <t>Independence level</t>
         </is>
       </c>
       <c r="C32" s="19" t="inlineStr"/>
@@ -1019,10 +1033,26 @@
     <row r="33" ht="18" customHeight="1">
       <c r="B33" s="18" t="inlineStr">
         <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C33" s="19" t="inlineStr"/>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="B34" s="18" t="inlineStr">
+        <is>
+          <t>Result (accepted / accepted with findings / rejected)</t>
+        </is>
+      </c>
+      <c r="C34" s="19" t="inlineStr"/>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="B35" s="18" t="inlineStr">
+        <is>
           <t>Findings reference</t>
         </is>
       </c>
-      <c r="C33" s="19" t="inlineStr"/>
+      <c r="C35" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8607,4 +8637,1337 @@
   <autoFilter ref="A1:E11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:P21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="5" customWidth="1" min="9" max="9"/>
+    <col width="5" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="30" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="54" t="inlineStr">
+        <is>
+          <t>FMEA-MSR (monitoring and system response, msr-plan.md): S, F, M and MSR AP per rating-tables.md §7 (RT-2). The MSR AP table is provisional until the handbook table is transcribed (decision register DQ-207). Exempt causes are rated in the FMEA named in the reason.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="28" t="inlineStr">
+        <is>
+          <t>Failure mode</t>
+        </is>
+      </c>
+      <c r="B2" s="29" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C2" s="29" t="inlineStr">
+        <is>
+          <t>Cause</t>
+        </is>
+      </c>
+      <c r="D2" s="28" t="inlineStr">
+        <is>
+          <t>Failure cause</t>
+        </is>
+      </c>
+      <c r="E2" s="28" t="inlineStr">
+        <is>
+          <t>Diagnostic</t>
+        </is>
+      </c>
+      <c r="F2" s="28" t="inlineStr">
+        <is>
+          <t>System response</t>
+        </is>
+      </c>
+      <c r="G2" s="28" t="inlineStr">
+        <is>
+          <t>Effect after the response</t>
+        </is>
+      </c>
+      <c r="H2" s="29" t="inlineStr">
+        <is>
+          <t>S after</t>
+        </is>
+      </c>
+      <c r="I2" s="29" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="J2" s="29" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="K2" s="29" t="inlineStr">
+        <is>
+          <t>MSR AP</t>
+        </is>
+      </c>
+      <c r="L2" s="28" t="inlineStr">
+        <is>
+          <t>Timing (FTTI · FDTI + FRTI)</t>
+        </is>
+      </c>
+      <c r="M2" s="29" t="inlineStr">
+        <is>
+          <t>Basis</t>
+        </is>
+      </c>
+      <c r="N2" s="28" t="inlineStr">
+        <is>
+          <t>Monitoring actions</t>
+        </is>
+      </c>
+      <c r="O2" s="28" t="inlineStr">
+        <is>
+          <t>Reviewer decision</t>
+        </is>
+      </c>
+      <c r="P2" s="28" t="inlineStr">
+        <is>
+          <t>Reviewer comment</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="46.5" customHeight="1">
+      <c r="A3" s="44" t="inlineStr">
+        <is>
+          <t>DFM-001 · Safety check computes a wrong result (permanent CPU or data-path fault)</t>
+        </is>
+      </c>
+      <c r="B3" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="C3" s="43" t="inlineStr">
+        <is>
+          <t>DFM-001.C1</t>
+        </is>
+      </c>
+      <c r="D3" s="44" t="inlineStr">
+        <is>
+          <t>Permanent fault in the Cortex-M7 core or bus matrix; single core, no lockstep, no CPU self-test</t>
+        </is>
+      </c>
+      <c r="E3" s="44" t="inlineStr">
+        <is>
+          <t>None in the MCU at BL-002. The host compares controls_allowed after about 2 s (QM); it does not check limits</t>
+        </is>
+      </c>
+      <c r="F3" s="44" t="inlineStr">
+        <is>
+          <t>None for a wrong limit result</t>
+        </is>
+      </c>
+      <c r="G3" s="44" t="inlineStr">
+        <is>
+          <t>Unchanged: a wrong check result lets an over-limit or unauthorised frame through</t>
+        </is>
+      </c>
+      <c r="H3" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="I3" s="45" t="n">
+        <v>6</v>
+      </c>
+      <c r="J3" s="46" t="n">
+        <v>9</v>
+      </c>
+      <c r="K3" s="47" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L3" s="44" t="inlineStr"/>
+      <c r="M3" s="43" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N3" s="44" t="inlineStr">
+        <is>
+          <t>DFM-ACT-001 · open</t>
+        </is>
+      </c>
+      <c r="O3" s="49" t="inlineStr"/>
+      <c r="P3" s="49" t="inlineStr"/>
+    </row>
+    <row r="4" ht="60" customHeight="1">
+      <c r="A4" s="44" t="inlineStr">
+        <is>
+          <t>DFM-002 · Code or limit constants corrupted in flash during operation</t>
+        </is>
+      </c>
+      <c r="B4" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="C4" s="43" t="inlineStr">
+        <is>
+          <t>DFM-002.C1</t>
+        </is>
+      </c>
+      <c r="D4" s="44" t="inlineStr">
+        <is>
+          <t>Multi-bit flash error or cell degradation; double-error ECC flag not handled; image signature checked at boot only</t>
+        </is>
+      </c>
+      <c r="E4" s="44" t="inlineStr">
+        <is>
+          <t>Bootstub signature check at power-up only; no periodic code CRC in the pinned firmware</t>
+        </is>
+      </c>
+      <c r="F4" s="44" t="inlineStr">
+        <is>
+          <t>None during the drive</t>
+        </is>
+      </c>
+      <c r="G4" s="44" t="inlineStr">
+        <is>
+          <t>Unchanged until the next power-up</t>
+        </is>
+      </c>
+      <c r="H4" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="I4" s="45" t="n">
+        <v>4</v>
+      </c>
+      <c r="J4" s="46" t="n">
+        <v>9</v>
+      </c>
+      <c r="K4" s="47" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L4" s="44" t="inlineStr"/>
+      <c r="M4" s="43" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N4" s="44" t="inlineStr">
+        <is>
+          <t>DFM-ACT-002 · open</t>
+        </is>
+      </c>
+      <c r="O4" s="49" t="inlineStr"/>
+      <c r="P4" s="49" t="inlineStr"/>
+    </row>
+    <row r="5" ht="46.5" customHeight="1">
+      <c r="A5" s="44" t="inlineStr">
+        <is>
+          <t>DFM-003 · Safety state in SRAM corrupted (controls_allowed, limits, counters, stack)</t>
+        </is>
+      </c>
+      <c r="B5" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="C5" s="43" t="inlineStr">
+        <is>
+          <t>DFM-003.C1</t>
+        </is>
+      </c>
+      <c r="D5" s="44" t="inlineStr">
+        <is>
+          <t>Double-bit soft error or permanent SRAM fault; RAMECC monitors not configured, ECC interrupt not registered</t>
+        </is>
+      </c>
+      <c r="E5" s="44" t="inlineStr">
+        <is>
+          <t>None at BL-002: RAMECC monitors not configured, no redundant storage</t>
+        </is>
+      </c>
+      <c r="F5" s="44" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G5" s="44" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="H5" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="I5" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="J5" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="K5" s="47" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L5" s="44" t="inlineStr"/>
+      <c r="M5" s="43" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N5" s="44" t="inlineStr">
+        <is>
+          <t>DFM-ACT-002 · open</t>
+        </is>
+      </c>
+      <c r="O5" s="49" t="inlineStr"/>
+      <c r="P5" s="49" t="inlineStr"/>
+    </row>
+    <row r="6" ht="46.5" customHeight="1">
+      <c r="A6" s="44" t="inlineStr">
+        <is>
+          <t>DFM-003 · Safety state in SRAM corrupted (controls_allowed, limits, counters, stack)</t>
+        </is>
+      </c>
+      <c r="B6" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="C6" s="43" t="inlineStr">
+        <is>
+          <t>DFM-003.C2</t>
+        </is>
+      </c>
+      <c r="D6" s="44" t="inlineStr">
+        <is>
+          <t>Wrong-address write by the SPI DMA (no MPU)</t>
+        </is>
+      </c>
+      <c r="E6" s="44" t="inlineStr">
+        <is>
+          <t>None at BL-002: no MPU and no redundant storage of the safety state</t>
+        </is>
+      </c>
+      <c r="F6" s="44" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G6" s="44" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="H6" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="I6" s="45" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="K6" s="47" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L6" s="44" t="inlineStr"/>
+      <c r="M6" s="43" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N6" s="44" t="inlineStr">
+        <is>
+          <t>DFM-ACT-002 · open</t>
+        </is>
+      </c>
+      <c r="O6" s="49" t="inlineStr"/>
+      <c r="P6" s="49" t="inlineStr"/>
+    </row>
+    <row r="7" ht="73.5" customHeight="1">
+      <c r="A7" s="44" t="inlineStr">
+        <is>
+          <t>DFM-004 · MCU execution stops with the relay energised</t>
+        </is>
+      </c>
+      <c r="B7" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="C7" s="43" t="inlineStr">
+        <is>
+          <t>DFM-004.C1</t>
+        </is>
+      </c>
+      <c r="D7" s="44" t="inlineStr">
+        <is>
+          <t>Hang in an ISR or main loop, unused vector to Default_Handler, or assert_fatal loop</t>
+        </is>
+      </c>
+      <c r="E7" s="44" t="inlineStr">
+        <is>
+          <t>IWDG expires about 90 ms after the last feed (T-09a). Timing fits on paper, but whether the reset releases the relay is unconfirmed (HWSR-502, UK-06) and the LSI tolerance leaves no shown margin (OI-7), so the response is not credited</t>
+        </is>
+      </c>
+      <c r="F7" s="44" t="inlineStr">
+        <is>
+          <t>MCU reset; relay de-energised if the drive circuit is de-energise-to-safe; stock camera CAN restored</t>
+        </is>
+      </c>
+      <c r="G7" s="44" t="inlineStr">
+        <is>
+          <t>Stock PCS/AEB restored and assist lost, if the relay releases</t>
+        </is>
+      </c>
+      <c r="H7" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="I7" s="45" t="n">
+        <v>6</v>
+      </c>
+      <c r="J7" s="45" t="n">
+        <v>7</v>
+      </c>
+      <c r="K7" s="47" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L7" s="44" t="inlineStr">
+        <is>
+          <t>SG-07 forwarding loss · 200 ms
+90 + 100 ms</t>
+        </is>
+      </c>
+      <c r="M7" s="43" t="inlineStr">
+        <is>
+          <t>code derived</t>
+        </is>
+      </c>
+      <c r="N7" s="44" t="inlineStr">
+        <is>
+          <t>DFM-ACT-003 · open</t>
+        </is>
+      </c>
+      <c r="O7" s="49" t="inlineStr"/>
+      <c r="P7" s="49" t="inlineStr"/>
+    </row>
+    <row r="8" ht="46.5" customHeight="1">
+      <c r="A8" s="44" t="inlineStr">
+        <is>
+          <t>DFM-007 · MCU operates in the brown-out zone</t>
+        </is>
+      </c>
+      <c r="B8" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="C8" s="43" t="inlineStr">
+        <is>
+          <t>DFM-007.C1</t>
+        </is>
+      </c>
+      <c r="D8" s="44" t="inlineStr">
+        <is>
+          <t>Vehicle supply dip (cranking, alternator fault) with BOR level not set and PVD not enabled</t>
+        </is>
+      </c>
+      <c r="E8" s="44" t="inlineStr">
+        <is>
+          <t>None at BL-002: PVD handler is a stub and the BOR level is unknown (UK-04)</t>
+        </is>
+      </c>
+      <c r="F8" s="44" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G8" s="44" t="inlineStr">
+        <is>
+          <t>Unchanged: erratic MCU behaviour in the brown-out zone</t>
+        </is>
+      </c>
+      <c r="H8" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="I8" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="K8" s="47" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L8" s="44" t="inlineStr"/>
+      <c r="M8" s="43" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N8" s="44" t="inlineStr">
+        <is>
+          <t>DFM-ACT-005 · open</t>
+        </is>
+      </c>
+      <c r="O8" s="49" t="inlineStr"/>
+      <c r="P8" s="49" t="inlineStr"/>
+    </row>
+    <row r="9" ht="46.5" customHeight="1">
+      <c r="A9" s="44" t="inlineStr">
+        <is>
+          <t>DFM-008 · Car-side transceiver holds the bus dominant</t>
+        </is>
+      </c>
+      <c r="B9" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="C9" s="43" t="inlineStr">
+        <is>
+          <t>DFM-008.C1</t>
+        </is>
+      </c>
+      <c r="D9" s="44" t="inlineStr">
+        <is>
+          <t>XCVR1 TX driver fault or TXD stuck low</t>
+        </is>
+      </c>
+      <c r="E9" s="44" t="inlineStr">
+        <is>
+          <t>FDCAN error counters; core reset on bus-off. The transceiver dominant timeout is part dependent and unknown</t>
+        </is>
+      </c>
+      <c r="F9" s="44" t="inlineStr">
+        <is>
+          <t>A core reset does not release a transceiver that holds the bus dominant; no safe-state reaction</t>
+        </is>
+      </c>
+      <c r="G9" s="44" t="inlineStr">
+        <is>
+          <t>Car bus blocked: loss of assist and of stock CAN functions until the transceiver times out, if it does</t>
+        </is>
+      </c>
+      <c r="H9" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="I9" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="J9" s="45" t="n">
+        <v>8</v>
+      </c>
+      <c r="K9" s="47" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L9" s="44" t="inlineStr"/>
+      <c r="M9" s="43" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N9" s="44" t="inlineStr">
+        <is>
+          <t>DFM-ACT-006 · open</t>
+        </is>
+      </c>
+      <c r="O9" s="49" t="inlineStr"/>
+      <c r="P9" s="49" t="inlineStr"/>
+    </row>
+    <row r="10" ht="46.5" customHeight="1">
+      <c r="A10" s="44" t="inlineStr">
+        <is>
+          <t>DFM-009 · Car-side transceiver receives nothing</t>
+        </is>
+      </c>
+      <c r="B10" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="C10" s="43" t="inlineStr">
+        <is>
+          <t>DFM-009.C1</t>
+        </is>
+      </c>
+      <c r="D10" s="44" t="inlineStr">
+        <is>
+          <t>XCVR1 RX open or stuck recessive</t>
+        </is>
+      </c>
+      <c r="E10" s="44" t="inlineStr">
+        <is>
+          <t>RX timeout after 5 periods (about 0.16 s) withdraws controls_allowed; the host warns through the 2 s controlsMismatch counter (T-17)</t>
+        </is>
+      </c>
+      <c r="F10" s="44" t="inlineStr">
+        <is>
+          <t>Authority withdrawn at once; warning about 2.2 s after onset, beyond the 1 s budget to warning</t>
+        </is>
+      </c>
+      <c r="G10" s="44" t="inlineStr">
+        <is>
+          <t>Assist lost; warning late</t>
+        </is>
+      </c>
+      <c r="H10" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="I10" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="J10" s="45" t="n">
+        <v>8</v>
+      </c>
+      <c r="K10" s="47" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L10" s="44" t="inlineStr">
+        <is>
+          <t>SG-02/06 loss without warning · 1000 ms
+160 + 2000 ms</t>
+        </is>
+      </c>
+      <c r="M10" s="43" t="inlineStr">
+        <is>
+          <t>code derived</t>
+        </is>
+      </c>
+      <c r="N10" s="44" t="inlineStr">
+        <is>
+          <t>DFM-ACT-006 · open</t>
+        </is>
+      </c>
+      <c r="O10" s="49" t="inlineStr"/>
+      <c r="P10" s="49" t="inlineStr"/>
+    </row>
+    <row r="11" ht="46.5" customHeight="1">
+      <c r="A11" s="44" t="inlineStr">
+        <is>
+          <t>DFM-010 · Intercept switch stays in intercept when released</t>
+        </is>
+      </c>
+      <c r="B11" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="43" t="inlineStr">
+        <is>
+          <t>DFM-010.C1</t>
+        </is>
+      </c>
+      <c r="D11" s="44" t="inlineStr">
+        <is>
+          <t>Analog switch U1 or U2 stuck in the intercept (NO) position, or its IN input damaged high</t>
+        </is>
+      </c>
+      <c r="E11" s="44" t="inlineStr">
+        <is>
+          <t>None: no relay readback (GAP-12)</t>
+        </is>
+      </c>
+      <c r="F11" s="44" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G11" s="44" t="inlineStr">
+        <is>
+          <t>Unchanged: stock camera stays cut off after release is commanded</t>
+        </is>
+      </c>
+      <c r="H11" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="I11" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="J11" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="K11" s="47" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L11" s="44" t="inlineStr"/>
+      <c r="M11" s="43" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N11" s="44" t="inlineStr">
+        <is>
+          <t>DFM-ACT-007 · open</t>
+        </is>
+      </c>
+      <c r="O11" s="49" t="inlineStr"/>
+      <c r="P11" s="49" t="inlineStr"/>
+    </row>
+    <row r="12" ht="46.5" customHeight="1">
+      <c r="A12" s="44" t="inlineStr">
+        <is>
+          <t>DFM-010 · Intercept switch stays in intercept when released</t>
+        </is>
+      </c>
+      <c r="B12" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="C12" s="43" t="inlineStr">
+        <is>
+          <t>DFM-010.C2</t>
+        </is>
+      </c>
+      <c r="D12" s="44" t="inlineStr">
+        <is>
+          <t>SBU1 drive stuck high (device-side driver or MCU pin, UK-06)</t>
+        </is>
+      </c>
+      <c r="E12" s="44" t="inlineStr">
+        <is>
+          <t>None: no relay readback (GAP-12)</t>
+        </is>
+      </c>
+      <c r="F12" s="44" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G12" s="44" t="inlineStr">
+        <is>
+          <t>Unchanged: stock camera stays cut off after release is commanded</t>
+        </is>
+      </c>
+      <c r="H12" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="I12" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="J12" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="K12" s="47" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L12" s="44" t="inlineStr"/>
+      <c r="M12" s="43" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N12" s="44" t="inlineStr">
+        <is>
+          <t>DFM-ACT-007 · open</t>
+        </is>
+      </c>
+      <c r="O12" s="49" t="inlineStr"/>
+      <c r="P12" s="49" t="inlineStr"/>
+    </row>
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="44" t="inlineStr">
+        <is>
+          <t>DFM-010 · Intercept switch stays in intercept when released</t>
+        </is>
+      </c>
+      <c r="B13" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="C13" s="43" t="inlineStr">
+        <is>
+          <t>DFM-010.C3</t>
+        </is>
+      </c>
+      <c r="D13" s="44" t="inlineStr">
+        <is>
+          <t>Pull-down R2 or R3 open, so IN floats when the device stops driving SBU1 (reset, watchdog, hang, unplugged cable)</t>
+        </is>
+      </c>
+      <c r="E13" s="44" t="inlineStr">
+        <is>
+          <t>None: the open pull-down is latent while the device drives SBU1, and no readback exists (GAP-12)</t>
+        </is>
+      </c>
+      <c r="F13" s="44" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G13" s="44" t="inlineStr">
+        <is>
+          <t>Unchanged: the switch may stay in intercept with the device silent, so the stock camera stays cut off</t>
+        </is>
+      </c>
+      <c r="H13" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="I13" s="45" t="n">
+        <v>2</v>
+      </c>
+      <c r="J13" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="K13" s="47" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L13" s="44" t="inlineStr"/>
+      <c r="M13" s="43" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N13" s="44" t="inlineStr">
+        <is>
+          <t>DFM-ACT-007 · open
+DFM-ACT-014 · open</t>
+        </is>
+      </c>
+      <c r="O13" s="49" t="inlineStr"/>
+      <c r="P13" s="49" t="inlineStr"/>
+    </row>
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="44" t="inlineStr">
+        <is>
+          <t>DFM-011 · Intercept switch stays in pass-through when driven</t>
+        </is>
+      </c>
+      <c r="B14" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="C14" s="43" t="inlineStr">
+        <is>
+          <t>DFM-011.C1</t>
+        </is>
+      </c>
+      <c r="D14" s="44" t="inlineStr">
+        <is>
+          <t>Analog switch U1 or U2 stuck in the pass-through (NC) position, or SBU1 drive lost or held low (driver open, R2/R3 short)</t>
+        </is>
+      </c>
+      <c r="E14" s="44" t="inlineStr">
+        <is>
+          <t>Relay malfunction: a stock camera frame on the car side after the 1 s grace blocks all TX (T-08, 1-2 s)</t>
+        </is>
+      </c>
+      <c r="F14" s="44" t="inlineStr">
+        <is>
+          <t>All TX blocked; host raises relayMalfunction (IMMEDIATE_DISABLE)</t>
+        </is>
+      </c>
+      <c r="G14" s="44" t="inlineStr">
+        <is>
+          <t>Up to 2 s of stock LKA and item commands on the bus together, then no item output</t>
+        </is>
+      </c>
+      <c r="H14" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="I14" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="J14" s="45" t="n">
+        <v>8</v>
+      </c>
+      <c r="K14" s="47" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L14" s="44" t="inlineStr">
+        <is>
+          <t>SG-01 relay stuck · 500 ms
+2000 + 10 ms</t>
+        </is>
+      </c>
+      <c r="M14" s="43" t="inlineStr">
+        <is>
+          <t>code derived</t>
+        </is>
+      </c>
+      <c r="N14" s="44" t="inlineStr">
+        <is>
+          <t>DFM-ACT-007 · open</t>
+        </is>
+      </c>
+      <c r="O14" s="49" t="inlineStr"/>
+      <c r="P14" s="49" t="inlineStr"/>
+    </row>
+    <row r="15" ht="46.5" customHeight="1">
+      <c r="A15" s="44" t="inlineStr">
+        <is>
+          <t>DFM-012 · Harness disconnected or intermittent while driving</t>
+        </is>
+      </c>
+      <c r="B15" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="C15" s="43" t="inlineStr">
+        <is>
+          <t>DFM-012.C1</t>
+        </is>
+      </c>
+      <c r="D15" s="44" t="inlineStr">
+        <is>
+          <t>Connector not fully latched at installation, or vibration loosens it</t>
+        </is>
+      </c>
+      <c r="E15" s="44" t="inlineStr">
+        <is>
+          <t>RX timeouts and host canBusMissing cover a partial disconnect only; a full disconnect also removes the device supply, so nothing warns</t>
+        </is>
+      </c>
+      <c r="F15" s="44" t="inlineStr">
+        <is>
+          <t>Relay drops out with the supply; stock camera restored</t>
+        </is>
+      </c>
+      <c r="G15" s="44" t="inlineStr">
+        <is>
+          <t>Assist lost without a LionDriver warning</t>
+        </is>
+      </c>
+      <c r="H15" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="I15" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="J15" s="46" t="n">
+        <v>9</v>
+      </c>
+      <c r="K15" s="47" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L15" s="44" t="inlineStr"/>
+      <c r="M15" s="43" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N15" s="44" t="inlineStr">
+        <is>
+          <t>DFM-ACT-008 · open</t>
+        </is>
+      </c>
+      <c r="O15" s="49" t="inlineStr"/>
+      <c r="P15" s="49" t="inlineStr"/>
+    </row>
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="44" t="inlineStr">
+        <is>
+          <t>DFM-016 · MCU forced into the ROM bootloader or reflashed by the SoC</t>
+        </is>
+      </c>
+      <c r="B16" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="C16" s="43" t="inlineStr">
+        <is>
+          <t>DFM-016.C1</t>
+        </is>
+      </c>
+      <c r="D16" s="44" t="inlineStr">
+        <is>
+          <t>SoC drives STM_BOOT0/STM_RST_N (fault or compromise); no RDP/WRP; pandad recovery flashes a development bootstub</t>
+        </is>
+      </c>
+      <c r="E16" s="44" t="inlineStr">
+        <is>
+          <t>Bootstub signature check exists but accepts the debug key in debug builds; RDP and WRP not set (GAP-24)</t>
+        </is>
+      </c>
+      <c r="F16" s="44" t="inlineStr">
+        <is>
+          <t>None for a signed debug image</t>
+        </is>
+      </c>
+      <c r="G16" s="44" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="H16" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="I16" s="45" t="n">
+        <v>4</v>
+      </c>
+      <c r="J16" s="46" t="n">
+        <v>9</v>
+      </c>
+      <c r="K16" s="47" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L16" s="44" t="inlineStr"/>
+      <c r="M16" s="43" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N16" s="44" t="inlineStr">
+        <is>
+          <t>DFM-ACT-010 · open</t>
+        </is>
+      </c>
+      <c r="O16" s="49" t="inlineStr"/>
+      <c r="P16" s="49" t="inlineStr"/>
+    </row>
+    <row r="17" ht="100.5" customHeight="1">
+      <c r="A17" s="44" t="inlineStr">
+        <is>
+          <t>DFM-019 · Approved CAN frame altered between the TX check and the bus</t>
+        </is>
+      </c>
+      <c r="B17" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="C17" s="43" t="inlineStr">
+        <is>
+          <t>DFM-019.C1</t>
+        </is>
+      </c>
+      <c r="D17" s="44" t="inlineStr">
+        <is>
+          <t>Soft error or permanent fault in the copy into FDCAN message RAM, the message RAM or the FDCAN core. The packet XOR is checked at the FDCAN load (fdcan.h:100) and covers only the software queue; the CAN CRC is computed after the fault</t>
+        </is>
+      </c>
+      <c r="E17" s="44" t="inlineStr">
+        <is>
+          <t>None after the FDCAN load: no TX read-back (TSR-517 not implemented)</t>
+        </is>
+      </c>
+      <c r="F17" s="44" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G17" s="44" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="H17" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="I17" s="45" t="n">
+        <v>4</v>
+      </c>
+      <c r="J17" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="K17" s="47" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L17" s="44" t="inlineStr"/>
+      <c r="M17" s="43" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N17" s="44" t="inlineStr">
+        <is>
+          <t>DFM-ACT-013 · open</t>
+        </is>
+      </c>
+      <c r="O17" s="49" t="inlineStr"/>
+      <c r="P17" s="49" t="inlineStr"/>
+    </row>
+    <row r="18" ht="100.5" customHeight="1">
+      <c r="A18" s="44" t="inlineStr">
+        <is>
+          <t>DFM-019 · Approved CAN frame altered between the TX check and the bus</t>
+        </is>
+      </c>
+      <c r="B18" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="C18" s="43" t="inlineStr">
+        <is>
+          <t>DFM-019.C2</t>
+        </is>
+      </c>
+      <c r="D18" s="44" t="inlineStr">
+        <is>
+          <t>Transceiver fault that changes bits on TX without a CAN error (not credible for a single bit, which the CAN CRC and the bit monitoring of the transmitting controller detect; kept until the transceiver part is known, WP-H-02 UK-01)</t>
+        </is>
+      </c>
+      <c r="E18" s="44" t="inlineStr">
+        <is>
+          <t>None: no TX read-back (TSR-517 not implemented)</t>
+        </is>
+      </c>
+      <c r="F18" s="44" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G18" s="44" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="H18" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="I18" s="45" t="n">
+        <v>2</v>
+      </c>
+      <c r="J18" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="K18" s="47" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L18" s="44" t="inlineStr"/>
+      <c r="M18" s="43" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N18" s="44" t="inlineStr">
+        <is>
+          <t>DFM-ACT-013 · open</t>
+        </is>
+      </c>
+      <c r="O18" s="49" t="inlineStr"/>
+      <c r="P18" s="49" t="inlineStr"/>
+    </row>
+    <row r="19" ht="46.5" customHeight="1">
+      <c r="A19" s="44" t="inlineStr">
+        <is>
+          <t>DFM-020 · Harness box loses its supply while the car is on</t>
+        </is>
+      </c>
+      <c r="B19" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="C19" s="43" t="inlineStr">
+        <is>
+          <t>DFM-020.C1</t>
+        </is>
+      </c>
+      <c r="D19" s="44" t="inlineStr">
+        <is>
+          <t>Ignition branch to the box open (crimp, connector) or D1 open, without comma power installed</t>
+        </is>
+      </c>
+      <c r="E19" s="44" t="inlineStr">
+        <is>
+          <t>None: the box supply is not supervised, and the device loses power with it</t>
+        </is>
+      </c>
+      <c r="F19" s="44" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G19" s="44" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="H19" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="I19" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="J19" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="K19" s="47" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L19" s="44" t="inlineStr"/>
+      <c r="M19" s="43" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N19" s="44" t="inlineStr">
+        <is>
+          <t>DFM-ACT-014 · open</t>
+        </is>
+      </c>
+      <c r="O19" s="49" t="inlineStr"/>
+      <c r="P19" s="49" t="inlineStr"/>
+    </row>
+    <row r="20" ht="33" customHeight="1">
+      <c r="A20" s="44" t="inlineStr">
+        <is>
+          <t>DFM-020 · Harness box loses its supply while the car is on</t>
+        </is>
+      </c>
+      <c r="B20" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="C20" s="43" t="inlineStr">
+        <is>
+          <t>DFM-020.C2</t>
+        </is>
+      </c>
+      <c r="D20" s="44" t="inlineStr">
+        <is>
+          <t>Box VIN shorted to ground (TVS D4 short, connector or wiring)</t>
+        </is>
+      </c>
+      <c r="E20" s="44" t="inlineStr">
+        <is>
+          <t>None: the box supply is not supervised, and the device loses power with it</t>
+        </is>
+      </c>
+      <c r="F20" s="44" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G20" s="44" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="H20" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="I20" s="45" t="n">
+        <v>3</v>
+      </c>
+      <c r="J20" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="K20" s="47" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L20" s="44" t="inlineStr"/>
+      <c r="M20" s="43" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N20" s="44" t="inlineStr">
+        <is>
+          <t>DFM-ACT-014 · open</t>
+        </is>
+      </c>
+      <c r="O20" s="49" t="inlineStr"/>
+      <c r="P20" s="49" t="inlineStr"/>
+    </row>
+    <row r="21" ht="46.5" customHeight="1">
+      <c r="A21" s="44" t="inlineStr">
+        <is>
+          <t>DFM-021 · Clamp diode short loads or grounds a vehicle bus in the harness box</t>
+        </is>
+      </c>
+      <c r="B21" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="C21" s="43" t="inlineStr">
+        <is>
+          <t>DFM-021.C1</t>
+        </is>
+      </c>
+      <c r="D21" s="44" t="inlineStr">
+        <is>
+          <t>Schottky clamp D2 or D3 (BAS40SDW) short or leaky</t>
+        </is>
+      </c>
+      <c r="E21" s="44" t="inlineStr">
+        <is>
+          <t>RX timeouts withdraw control and the host raises CAN errors; nothing restores the bus</t>
+        </is>
+      </c>
+      <c r="F21" s="44" t="inlineStr">
+        <is>
+          <t>Authority withdrawn and the driver warned; the stock camera path stays broken</t>
+        </is>
+      </c>
+      <c r="G21" s="44" t="inlineStr">
+        <is>
+          <t>Item disengaged, but stock AEB stays unavailable</t>
+        </is>
+      </c>
+      <c r="H21" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="I21" s="45" t="n">
+        <v>3</v>
+      </c>
+      <c r="J21" s="45" t="n">
+        <v>8</v>
+      </c>
+      <c r="K21" s="47" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L21" s="44" t="inlineStr"/>
+      <c r="M21" s="43" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N21" s="44" t="inlineStr">
+        <is>
+          <t>DFM-ACT-014 · open</t>
+        </is>
+      </c>
+      <c r="O21" s="49" t="inlineStr"/>
+      <c r="P21" s="49" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:P21"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:P1"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="O3 O4 O5 O6 O7 O8 O9 O10 O11 O12 O13 O14 O15 O16 O17 O18 O19 O20 O21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this MSR row" type="list">
+      <formula1>"Agree,Re-rate,Reject,Question"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;LDFMEA — device, integrated panda, harness, vehicle interfaces · FMEA-MSR · rev 0.5 · BL-002&amp;RPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Apply DQ-209 option A: keep comma's harness box and bench-test it
- WP-H-01 v0.9: HWSR-702 decided (deviation, bench-tested, assumption of
  use); HWSR-506a no readback planned; HWSR-506e route; OI-6.
- WP-H-02 v0.9: OI-4, DC-03 not pursued.
- WP-H-06 v0.7: VS-HW-02, -22..24 are the decided route (spare box).
- RR-2026-010 §5: decision recorded.
- DFMEA: DFM-ACT-007 not_implemented; DFM-ACT-014 is the route.
- Register: DQ-209 applied; DQ-261 queued (accept the SG-07 SPFM
  shortfall of 78.1 % vs 90 % as a recorded deviation?).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xx6vAdwvGpomGg8X6smJDx
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/dfmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/dfmea-review.xlsx
@@ -3794,7 +3794,7 @@
       <c r="R12" s="39" t="inlineStr"/>
       <c r="S12" s="39" t="inlineStr"/>
     </row>
-    <row r="13" ht="87" customHeight="1">
+    <row r="13" ht="127.5" customHeight="1">
       <c r="A13" s="40" t="inlineStr">
         <is>
           <r>
@@ -4022,13 +4022,13 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Add relay readback in a LionDriver harness adapter (WP-H-02 DC-03) and confirm the de-energised contact state (UK-03)</t>
+            <t>Add relay readback in a LionDriver harness adapter (WP-H-02 DC-03) and confirm the de-energised contact state (UK-03). Not implemented by decision DQ-209 option A (2026-10-16): comma's box is kept and its failure behaviour is bench-tested (DFM-ACT-014) and argued as residual risk; the de-energised state is covered by DFM-ACT-014</t>
           </r>
         </is>
       </c>
       <c r="O13" s="48" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not implemented</t>
         </is>
       </c>
       <c r="P13" s="43" t="inlineStr"/>
@@ -4036,7 +4036,7 @@
       <c r="R13" s="49" t="inlineStr"/>
       <c r="S13" s="49" t="inlineStr"/>
     </row>
-    <row r="14" ht="87" customHeight="1">
+    <row r="14" ht="127.5" customHeight="1">
       <c r="A14" s="51" t="n"/>
       <c r="B14" s="51" t="n"/>
       <c r="C14" s="51" t="n"/>
@@ -4122,13 +4122,13 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Add relay readback in a LionDriver harness adapter (WP-H-02 DC-03) and confirm the de-energised contact state (UK-03)</t>
+            <t>Add relay readback in a LionDriver harness adapter (WP-H-02 DC-03) and confirm the de-energised contact state (UK-03). Not implemented by decision DQ-209 option A (2026-10-16): comma's box is kept and its failure behaviour is bench-tested (DFM-ACT-014) and argued as residual risk; the de-energised state is covered by DFM-ACT-014</t>
           </r>
         </is>
       </c>
       <c r="O14" s="48" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not implemented</t>
         </is>
       </c>
       <c r="P14" s="43" t="inlineStr"/>
@@ -4136,7 +4136,7 @@
       <c r="R14" s="49" t="inlineStr"/>
       <c r="S14" s="49" t="inlineStr"/>
     </row>
-    <row r="15" ht="181.5" customHeight="1">
+    <row r="15" ht="276" customHeight="1">
       <c r="A15" s="51" t="n"/>
       <c r="B15" s="51" t="n"/>
       <c r="C15" s="51" t="n"/>
@@ -4222,7 +4222,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Add relay readback in a LionDriver harness adapter (WP-H-02 DC-03) and confirm the de-energised contact state (UK-03)</t>
+            <t>Add relay readback in a LionDriver harness adapter (WP-H-02 DC-03) and confirm the de-energised contact state (UK-03). Not implemented by decision DQ-209 option A (2026-10-16): comma's box is kept and its failure behaviour is bench-tested (DFM-ACT-014) and argued as residual risk; the de-energised state is covered by DFM-ACT-014</t>
           </r>
           <r>
             <rPr>
@@ -4249,13 +4249,13 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02)</t>
+            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
           </r>
         </is>
       </c>
       <c r="O15" s="48" t="inlineStr">
         <is>
-          <t>open
+          <t>not implemented
 open</t>
         </is>
       </c>
@@ -4264,7 +4264,7 @@
       <c r="R15" s="49" t="inlineStr"/>
       <c r="S15" s="49" t="inlineStr"/>
     </row>
-    <row r="16" ht="276" customHeight="1">
+    <row r="16" ht="303" customHeight="1">
       <c r="A16" s="50" t="n"/>
       <c r="B16" s="50" t="n"/>
       <c r="C16" s="50" t="n"/>
@@ -4376,7 +4376,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02)</t>
+            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
           </r>
           <r>
             <rPr>
@@ -4418,7 +4418,7 @@
       <c r="R16" s="39" t="inlineStr"/>
       <c r="S16" s="39" t="inlineStr"/>
     </row>
-    <row r="17" ht="87" customHeight="1">
+    <row r="17" ht="127.5" customHeight="1">
       <c r="A17" s="40" t="inlineStr">
         <is>
           <r>
@@ -4682,13 +4682,13 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Add relay readback in a LionDriver harness adapter (WP-H-02 DC-03) and confirm the de-energised contact state (UK-03)</t>
+            <t>Add relay readback in a LionDriver harness adapter (WP-H-02 DC-03) and confirm the de-energised contact state (UK-03). Not implemented by decision DQ-209 option A (2026-10-16): comma's box is kept and its failure behaviour is bench-tested (DFM-ACT-014) and argued as residual risk; the de-energised state is covered by DFM-ACT-014</t>
           </r>
         </is>
       </c>
       <c r="O17" s="48" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not implemented</t>
         </is>
       </c>
       <c r="P17" s="43" t="inlineStr"/>
@@ -4696,7 +4696,7 @@
       <c r="R17" s="49" t="inlineStr"/>
       <c r="S17" s="49" t="inlineStr"/>
     </row>
-    <row r="18" ht="276" customHeight="1">
+    <row r="18" ht="303" customHeight="1">
       <c r="A18" s="50" t="n"/>
       <c r="B18" s="50" t="n"/>
       <c r="C18" s="50" t="n"/>
@@ -4817,7 +4817,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02)</t>
+            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
           </r>
           <r>
             <rPr>
@@ -5585,7 +5585,7 @@
       <c r="R21" s="49" t="inlineStr"/>
       <c r="S21" s="49" t="inlineStr"/>
     </row>
-    <row r="22" ht="181.5" customHeight="1">
+    <row r="22" ht="208.5" customHeight="1">
       <c r="A22" s="50" t="n"/>
       <c r="B22" s="50" t="n"/>
       <c r="C22" s="50" t="n"/>
@@ -5698,7 +5698,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02)</t>
+            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
           </r>
         </is>
       </c>
@@ -7336,7 +7336,7 @@
       <c r="R29" s="39" t="inlineStr"/>
       <c r="S29" s="39" t="inlineStr"/>
     </row>
-    <row r="30" ht="127.5" customHeight="1">
+    <row r="30" ht="154.5" customHeight="1">
       <c r="A30" s="40" t="inlineStr">
         <is>
           <r>
@@ -7591,7 +7591,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02)</t>
+            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
           </r>
         </is>
       </c>
@@ -7605,7 +7605,7 @@
       <c r="R30" s="49" t="inlineStr"/>
       <c r="S30" s="49" t="inlineStr"/>
     </row>
-    <row r="31" ht="127.5" customHeight="1">
+    <row r="31" ht="154.5" customHeight="1">
       <c r="A31" s="50" t="n"/>
       <c r="B31" s="50" t="n"/>
       <c r="C31" s="50" t="n"/>
@@ -7691,7 +7691,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02)</t>
+            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
           </r>
         </is>
       </c>
@@ -7705,7 +7705,7 @@
       <c r="R31" s="39" t="inlineStr"/>
       <c r="S31" s="39" t="inlineStr"/>
     </row>
-    <row r="32" ht="127.5" customHeight="1">
+    <row r="32" ht="154.5" customHeight="1">
       <c r="A32" s="30" t="inlineStr">
         <is>
           <r>
@@ -7960,7 +7960,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02)</t>
+            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
           </r>
         </is>
       </c>
@@ -8323,7 +8323,7 @@
       <c r="H7" s="53" t="inlineStr"/>
       <c r="I7" s="53" t="inlineStr"/>
     </row>
-    <row r="8" ht="60" customHeight="1">
+    <row r="8" ht="73.5" customHeight="1">
       <c r="A8" s="53" t="inlineStr">
         <is>
           <t>DFM-ACT-007</t>
@@ -8336,7 +8336,7 @@
       </c>
       <c r="C8" s="53" t="inlineStr">
         <is>
-          <t>Add relay readback in a LionDriver harness adapter (WP-H-02 DC-03) and confirm the de-energised contact state (UK-03)</t>
+          <t>Add relay readback in a LionDriver harness adapter (WP-H-02 DC-03) and confirm the de-energised contact state (UK-03). Not implemented by decision DQ-209 option A (2026-10-16): comma's box is kept and its failure behaviour is bench-tested (DFM-ACT-014) and argued as residual risk; the de-energised state is covered by DFM-ACT-014</t>
         </is>
       </c>
       <c r="D8" s="53" t="inlineStr">
@@ -8346,7 +8346,7 @@
       </c>
       <c r="E8" s="53" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>not implemented</t>
         </is>
       </c>
       <c r="F8" s="53" t="inlineStr">
@@ -8589,7 +8589,7 @@
       </c>
       <c r="C15" s="53" t="inlineStr">
         <is>
-          <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02)</t>
+          <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
         </is>
       </c>
       <c r="D15" s="53" t="inlineStr">

</xml_diff>

<commit_message>
DFMEA rev 0.8: EPS-fault siren persistence 0.7 s (DQ-048, panda bf8102a)
DFM-017 mechanism text: the siren sounds after a 0.7 s persistent EPS fault,
at most 0.96 s after onset by design (WP-S-04 T-28; was 1 s / 1.26 s).
New action DFM-ACT-016: time the chain on the HIL bench (margin 0.04 s),
waiting for the bench (DQ-049). Ratings unchanged. fmea-plan and msr-plan
summary lines updated; review pages and figures regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xx6vAdwvGpomGg8X6smJDx
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/dfmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/dfmea-review.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$32</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Worksheet'!$1:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Structure'!$A$1:$E$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'MSR'!$A$2:$P$25</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'MSR'!$1:$2</definedName>
@@ -787,7 +787,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.7 · draft</t>
+          <t>0.8 · draft</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>15 (15)</t>
+          <t>16 (16)</t>
         </is>
       </c>
     </row>
@@ -6280,7 +6280,7 @@
       <c r="R24" s="39" t="inlineStr"/>
       <c r="S24" s="39" t="inlineStr"/>
     </row>
-    <row r="25" ht="87" customHeight="1">
+    <row r="25" ht="208.5" customHeight="1">
       <c r="A25" s="40" t="inlineStr">
         <is>
           <r>
@@ -6537,11 +6537,39 @@
             </rPr>
             <t>Confirm the siren audio topology (UK-07) and add a start-up siren self-test (TSR-515/516)</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">DFM-ACT-016 · detection
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Time the EPS-fault warning chain on the HIL bench (WP-S-04 T-28): inject a persistent LKA_STATE fault on 0x262 while authority is granted and measure fault onset to audible siren against the 0.96 s design worst case and the SG-02 1 s budget (margin 0.04 s), with the speaker phase varied. Persistence 0.7 s since panda bf8102a (DQ-048). Waits for the HIL bench, which the lead deferred (DQ-049, 2026-10-14)</t>
+          </r>
         </is>
       </c>
       <c r="O25" s="48" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>open
+open</t>
         </is>
       </c>
       <c r="P25" s="43" t="inlineStr"/>
@@ -6549,7 +6577,7 @@
       <c r="R25" s="49" t="inlineStr"/>
       <c r="S25" s="49" t="inlineStr"/>
     </row>
-    <row r="26" ht="87" customHeight="1">
+    <row r="26" ht="208.5" customHeight="1">
       <c r="A26" s="50" t="n"/>
       <c r="B26" s="50" t="n"/>
       <c r="C26" s="50" t="n"/>
@@ -6637,11 +6665,39 @@
             </rPr>
             <t>Confirm the siren audio topology (UK-07) and add a start-up siren self-test (TSR-515/516)</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">DFM-ACT-016 · detection
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Time the EPS-fault warning chain on the HIL bench (WP-S-04 T-28): inject a persistent LKA_STATE fault on 0x262 while authority is granted and measure fault onset to audible siren against the 0.96 s design worst case and the SG-02 1 s budget (margin 0.04 s), with the speaker phase varied. Persistence 0.7 s since panda bf8102a (DQ-048). Waits for the HIL bench, which the lead deferred (DQ-049, 2026-10-14)</t>
+          </r>
         </is>
       </c>
       <c r="O26" s="38" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>open
+open</t>
         </is>
       </c>
       <c r="P26" s="33" t="inlineStr"/>
@@ -8063,7 +8119,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LDFMEA — device, integrated panda, harness, vehicle interfaces · rev 0.7 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LDFMEA — device, integrated panda, harness, vehicle interfaces · rev 0.8 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -8078,7 +8134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8683,8 +8739,44 @@
       <c r="H16" s="53" t="inlineStr"/>
       <c r="I16" s="53" t="inlineStr"/>
     </row>
+    <row r="17" ht="87" customHeight="1">
+      <c r="A17" s="53" t="inlineStr">
+        <is>
+          <t>DFM-ACT-016</t>
+        </is>
+      </c>
+      <c r="B17" s="53" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="C17" s="53" t="inlineStr">
+        <is>
+          <t>Time the EPS-fault warning chain on the HIL bench (WP-S-04 T-28): inject a persistent LKA_STATE fault on 0x262 while authority is granted and measure fault onset to audible siren against the 0.96 s design worst case and the SG-02 1 s budget (margin 0.04 s), with the speaker phase varied. Persistence 0.7 s since panda bf8102a (DQ-048). Waits for the HIL bench, which the lead deferred (DQ-049, 2026-10-14)</t>
+        </is>
+      </c>
+      <c r="D17" s="53" t="inlineStr">
+        <is>
+          <t>Jherrod Thomas</t>
+        </is>
+      </c>
+      <c r="E17" s="53" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="F17" s="53" t="inlineStr">
+        <is>
+          <t>DFM-017.C1
+DFM-017.C2</t>
+        </is>
+      </c>
+      <c r="G17" s="53" t="inlineStr"/>
+      <c r="H17" s="53" t="inlineStr"/>
+      <c r="I17" s="53" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I16"/>
+  <autoFilter ref="A1:I17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10187,7 +10279,8 @@
       </c>
       <c r="N19" s="44" t="inlineStr">
         <is>
-          <t>DFM-ACT-011 · open</t>
+          <t>DFM-ACT-011 · open
+DFM-ACT-016 · open</t>
         </is>
       </c>
       <c r="O19" s="49" t="inlineStr"/>
@@ -10249,7 +10342,8 @@
       </c>
       <c r="N20" s="44" t="inlineStr">
         <is>
-          <t>DFM-ACT-011 · open</t>
+          <t>DFM-ACT-011 · open
+DFM-ACT-016 · open</t>
         </is>
       </c>
       <c r="O20" s="49" t="inlineStr"/>
@@ -10579,7 +10673,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LDFMEA — device, integrated panda, harness, vehicle interfaces · FMEA-MSR · rev 0.7 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LDFMEA — device, integrated panda, harness, vehicle interfaces · FMEA-MSR · rev 0.8 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
DFMEA rev 0.13: harness box camera-side termination R7/R8 in intercept
FMEDA SG-009 rev 0.9 (#511) added R7/R8 (FMD-C-014) with no DFMEA row.
New rows, both S 10 for HZ-011 (stock AEB unavailable):
- DFM-022, camera bus unterminated in intercept: R7 with R8 or the
  P13-P15 loopback open. One open alone is latent. The SPICE pilot
  (#510) predicts a 10.5 us recessive edge with both gone. O 2 D 10 AP H;
  MSR F 2 M 10 AP M.
- DFM-023, R7 or R8 short, camera bus held recessive. O 3 D 10 AP H;
  MSR F 3 M 10 AP H.
DFM-ACT-014 now names the VS-HW-24 (e) bench step. fta-fmea-map records
both as SG-07 tree gaps for the FTA owner. fmea-plan v0.37. DFMEA
review page, workbook, figures and the workbook viewer fingerprint
regenerated. The FMEDA dfmea_ref links are left to the FMEDA owner.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LcRUDDo8nS295kJpM99msk
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/dfmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/dfmea-review.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MSR" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Worksheet'!$1:$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Structure'!$A$1:$E$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'MSR'!$A$2:$P$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'MSR'!$A$2:$P$27</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'MSR'!$1:$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -790,7 +790,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.12 · draft</t>
+          <t>0.13 · draft</t>
         </is>
       </c>
     </row>
@@ -868,7 +868,7 @@
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="15">
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="C15" s="8" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16">
@@ -888,7 +888,7 @@
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17">
@@ -931,7 +931,7 @@
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>23 rated, 0 exempt; MSR AP H 20, M 3, L 0</t>
+          <t>25 rated, 0 exempt; MSR AP H 21, M 4, L 0</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>1–4: 0 · 5–6: 1 · 7–8: 5 · 9–10: 17 (see sheet MSR)</t>
+          <t>1–4: 0 · 5–6: 1 · 7–8: 5 · 9–10: 19 (see sheet MSR)</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S32"/>
+  <dimension ref="A1:S34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4169,7 +4169,7 @@
       <c r="R14" s="49" t="inlineStr"/>
       <c r="S14" s="49" t="inlineStr"/>
     </row>
-    <row r="15" ht="276" customHeight="1">
+    <row r="15" ht="303" customHeight="1">
       <c r="A15" s="51" t="n"/>
       <c r="B15" s="51" t="n"/>
       <c r="C15" s="51" t="n"/>
@@ -4282,7 +4282,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
+            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; camera-side termination R7/R8 lifted in intercept (VS-HW-24 (e), DFM-022); confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
           </r>
         </is>
       </c>
@@ -4297,7 +4297,7 @@
       <c r="R15" s="49" t="inlineStr"/>
       <c r="S15" s="49" t="inlineStr"/>
     </row>
-    <row r="16" ht="303" customHeight="1">
+    <row r="16" ht="330" customHeight="1">
       <c r="A16" s="50" t="n"/>
       <c r="B16" s="50" t="n"/>
       <c r="C16" s="50" t="n"/>
@@ -4409,7 +4409,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
+            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; camera-side termination R7/R8 lifted in intercept (VS-HW-24 (e), DFM-022); confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
           </r>
           <r>
             <rPr>
@@ -4729,7 +4729,7 @@
       <c r="R17" s="49" t="inlineStr"/>
       <c r="S17" s="49" t="inlineStr"/>
     </row>
-    <row r="18" ht="303" customHeight="1">
+    <row r="18" ht="330" customHeight="1">
       <c r="A18" s="50" t="n"/>
       <c r="B18" s="50" t="n"/>
       <c r="C18" s="50" t="n"/>
@@ -4850,7 +4850,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
+            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; camera-side termination R7/R8 lifted in intercept (VS-HW-24 (e), DFM-022); confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
           </r>
           <r>
             <rPr>
@@ -5618,7 +5618,7 @@
       <c r="R21" s="49" t="inlineStr"/>
       <c r="S21" s="49" t="inlineStr"/>
     </row>
-    <row r="22" ht="208.5" customHeight="1">
+    <row r="22" ht="235.5" customHeight="1">
       <c r="A22" s="50" t="n"/>
       <c r="B22" s="50" t="n"/>
       <c r="C22" s="50" t="n"/>
@@ -5731,7 +5731,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
+            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; camera-side termination R7/R8 lifted in intercept (VS-HW-24 (e), DFM-022); confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
           </r>
         </is>
       </c>
@@ -7425,7 +7425,7 @@
       <c r="R29" s="39" t="inlineStr"/>
       <c r="S29" s="39" t="inlineStr"/>
     </row>
-    <row r="30" ht="154.5" customHeight="1">
+    <row r="30" ht="181.5" customHeight="1">
       <c r="A30" s="40" t="inlineStr">
         <is>
           <r>
@@ -7680,7 +7680,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
+            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; camera-side termination R7/R8 lifted in intercept (VS-HW-24 (e), DFM-022); confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
           </r>
         </is>
       </c>
@@ -7694,7 +7694,7 @@
       <c r="R30" s="49" t="inlineStr"/>
       <c r="S30" s="49" t="inlineStr"/>
     </row>
-    <row r="31" ht="154.5" customHeight="1">
+    <row r="31" ht="181.5" customHeight="1">
       <c r="A31" s="50" t="n"/>
       <c r="B31" s="50" t="n"/>
       <c r="C31" s="50" t="n"/>
@@ -7780,7 +7780,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
+            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; camera-side termination R7/R8 lifted in intercept (VS-HW-24 (e), DFM-022); confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
           </r>
         </is>
       </c>
@@ -7794,7 +7794,7 @@
       <c r="R31" s="39" t="inlineStr"/>
       <c r="S31" s="39" t="inlineStr"/>
     </row>
-    <row r="32" ht="154.5" customHeight="1">
+    <row r="32" ht="181.5" customHeight="1">
       <c r="A32" s="30" t="inlineStr">
         <is>
           <r>
@@ -8049,7 +8049,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
+            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; camera-side termination R7/R8 lifted in intercept (VS-HW-24 (e), DFM-022); confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
           </r>
         </is>
       </c>
@@ -8063,8 +8063,501 @@
       <c r="R32" s="39" t="inlineStr"/>
       <c r="S32" s="39" t="inlineStr"/>
     </row>
+    <row r="33" ht="181.5" customHeight="1">
+      <c r="A33" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">DFM-SE-006
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Intercept switch (harness box U1/U2) and its drive</t>
+          </r>
+        </is>
+      </c>
+      <c r="B33" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">DFM-FN-005
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Separate the camera from the car bus only while energised; restore the stock camera path whenever de-energised</t>
+          </r>
+        </is>
+      </c>
+      <c r="C33" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Stock AEB unavailable</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">Next higher  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Camera frames lost or corrupted while the device forwards them, so stock PCS messages do not reach the car</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">Local  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>In intercept only the box terminates the camera bus (R7, and R8 through the harness P13-P15 loopback, 60 ohm). With both gone the recessive edge slows to about 10.5 us and misses the 1.5 us sample point (harness box SPICE pilot, a prediction)</t>
+          </r>
+        </is>
+      </c>
+      <c r="D33" s="31" t="inlineStr">
+        <is>
+          <t>HZ-011</t>
+        </is>
+      </c>
+      <c r="E33" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="F33" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">DFM-022 · open
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Camera bus left unterminated in intercept</t>
+          </r>
+        </is>
+      </c>
+      <c r="G33" s="33" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Termination resistor R7 open together with R8 or the P13-P15 loopback open. One open alone leaves 120 ohm and a recessive edge of about 0.06 us, so it is latent (FMEDA SG-009 FMD-035); pass-through is not affected (R7/R8 are on the NO side)</t>
+          </r>
+        </is>
+      </c>
+      <c r="I33" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• COTS comma 3X design in volume field use; no supplier reliability data, schematic or BOM available to LionDriver (WP-H-02 UK-01, UK-02)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   assurance/04-hardware/WP-H-02-hardware-design.md</t>
+          </r>
+        </is>
+      </c>
+      <c r="J33" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="K33" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• No LionDriver hardware test has been run for this cause. Bench step VS-HW-24 (e) lifts R7, R8, then both, in intercept and records error frames and the recessive edge (WP-H-06 v0.13); not yet run</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   assurance/04-hardware/WP-H-06-hardware-integration-verification.md</t>
+          </r>
+        </is>
+      </c>
+      <c r="L33" s="36" t="n">
+        <v>10</v>
+      </c>
+      <c r="M33" s="37" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="N33" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">DFM-ACT-014 · detection
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; camera-side termination R7/R8 lifted in intercept (VS-HW-24 (e), DFM-022); confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
+          </r>
+        </is>
+      </c>
+      <c r="O33" s="38" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="P33" s="33" t="inlineStr"/>
+      <c r="Q33" s="33" t="inlineStr"/>
+      <c r="R33" s="39" t="inlineStr"/>
+      <c r="S33" s="39" t="inlineStr"/>
+    </row>
+    <row r="34" ht="181.5" customHeight="1">
+      <c r="A34" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">DFM-SE-006
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Intercept switch (harness box U1/U2) and its drive</t>
+          </r>
+        </is>
+      </c>
+      <c r="B34" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">DFM-FN-005
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Separate the camera from the car bus only while energised; restore the stock camera path whenever de-energised</t>
+          </r>
+        </is>
+      </c>
+      <c r="C34" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Stock AEB unavailable</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">Next higher  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>No camera frames reach the device, so stock PCS messages are not forwarded to the car</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">Local  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>R7 or R8 short ties camera CAN2_H to CAN2_L, so the camera bus is held recessive in intercept</t>
+          </r>
+        </is>
+      </c>
+      <c r="D34" s="31" t="inlineStr">
+        <is>
+          <t>HZ-011</t>
+        </is>
+      </c>
+      <c r="E34" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="F34" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">DFM-023 · short
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Camera-side termination shorted in intercept</t>
+          </r>
+        </is>
+      </c>
+      <c r="G34" s="33" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Termination resistor R7 or R8 short (FMEDA SG-009 FMD-036); pass-through is not affected (R7/R8 are on the NO side)</t>
+          </r>
+        </is>
+      </c>
+      <c r="I34" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• COTS comma 3X design in volume field use; no supplier reliability data, schematic or BOM available to LionDriver (WP-H-02 UK-01, UK-02)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   assurance/04-hardware/WP-H-02-hardware-design.md</t>
+          </r>
+        </is>
+      </c>
+      <c r="J34" s="35" t="n">
+        <v>3</v>
+      </c>
+      <c r="K34" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• No LionDriver hardware verification or qualification test exists for this cause; VS-HW-24 (e) checks the opens only (WP-H-06 v0.13)</t>
+          </r>
+        </is>
+      </c>
+      <c r="L34" s="36" t="n">
+        <v>10</v>
+      </c>
+      <c r="M34" s="37" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="N34" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">DFM-ACT-014 · detection
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; camera-side termination R7/R8 lifted in intercept (VS-HW-24 (e), DFM-022); confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
+          </r>
+        </is>
+      </c>
+      <c r="O34" s="38" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="P34" s="33" t="inlineStr"/>
+      <c r="Q34" s="33" t="inlineStr"/>
+      <c r="R34" s="39" t="inlineStr"/>
+      <c r="S34" s="39" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:S32"/>
+  <autoFilter ref="A2:S34"/>
   <mergeCells count="46">
     <mergeCell ref="C30:C31"/>
     <mergeCell ref="E5:E6"/>
@@ -8114,7 +8607,7 @@
     <mergeCell ref="C5:C6"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="R3 R4 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this cause" type="list">
+    <dataValidation sqref="R3 R4 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32 R33 R34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this cause" type="list">
       <formula1>"Agree,Re-rate,Reject,Question"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8122,7 +8615,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LDFMEA — device, integrated panda, harness, vehicle interfaces · rev 0.12 · BL-007&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LDFMEA — device, integrated panda, harness, vehicle interfaces · rev 0.13 · BL-007&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -8665,7 +9158,7 @@
       <c r="H14" s="53" t="inlineStr"/>
       <c r="I14" s="53" t="inlineStr"/>
     </row>
-    <row r="15" ht="100.5" customHeight="1">
+    <row r="15" ht="127.5" customHeight="1">
       <c r="A15" s="53" t="inlineStr">
         <is>
           <t>DFM-ACT-014</t>
@@ -8678,7 +9171,7 @@
       </c>
       <c r="C15" s="53" t="inlineStr">
         <is>
-          <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
+          <t>Bench-test the harness box failure behaviour (RR-2026-010): box unpowered with car and camera powered; R2/R3 forced open with the device silent; supply at 14-16 V against the DG419LE ratings; pass-through signal integrity; clamp-diode short on CAN0; camera-side termination R7/R8 lifted in intercept (VS-HW-24 (e), DFM-022); confirm the shipped box matches the v3 drawing (VS-HW-02). The decided route for the harness box (DQ-209 option A, 2026-10-16); procedures in WP-H-06 §3.1</t>
         </is>
       </c>
       <c r="D15" s="53" t="inlineStr">
@@ -8699,7 +9192,9 @@
 DFM-014.C2
 DFM-020.C1
 DFM-020.C2
-DFM-021.C1</t>
+DFM-021.C1
+DFM-022.C1
+DFM-023.C1</t>
         </is>
       </c>
       <c r="G15" s="53" t="inlineStr"/>
@@ -9101,7 +9596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -10662,13 +11157,137 @@
       <c r="O25" s="49" t="inlineStr"/>
       <c r="P25" s="49" t="inlineStr"/>
     </row>
+    <row r="26" ht="100.5" customHeight="1">
+      <c r="A26" s="44" t="inlineStr">
+        <is>
+          <t>DFM-022 · Camera bus left unterminated in intercept</t>
+        </is>
+      </c>
+      <c r="B26" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="C26" s="43" t="inlineStr">
+        <is>
+          <t>DFM-022.C1</t>
+        </is>
+      </c>
+      <c r="D26" s="44" t="inlineStr">
+        <is>
+          <t>Termination resistor R7 open together with R8 or the P13-P15 loopback open. One open alone leaves 120 ohm and a recessive edge of about 0.06 us, so it is latent (FMEDA SG-009 FMD-035); pass-through is not affected (R7/R8 are on the NO side)</t>
+        </is>
+      </c>
+      <c r="E26" s="44" t="inlineStr">
+        <is>
+          <t>None: the device checks only car-side messages for timeouts; a single open is latent and nothing checks the camera-side termination</t>
+        </is>
+      </c>
+      <c r="F26" s="44" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G26" s="44" t="inlineStr">
+        <is>
+          <t>Unchanged: stock PCS messages are lost while in intercept</t>
+        </is>
+      </c>
+      <c r="H26" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="I26" s="45" t="n">
+        <v>2</v>
+      </c>
+      <c r="J26" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="K26" s="55" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="L26" s="44" t="inlineStr"/>
+      <c r="M26" s="43" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N26" s="44" t="inlineStr">
+        <is>
+          <t>DFM-ACT-014 · open</t>
+        </is>
+      </c>
+      <c r="O26" s="49" t="inlineStr"/>
+      <c r="P26" s="49" t="inlineStr"/>
+    </row>
+    <row r="27" ht="60" customHeight="1">
+      <c r="A27" s="44" t="inlineStr">
+        <is>
+          <t>DFM-023 · Camera-side termination shorted in intercept</t>
+        </is>
+      </c>
+      <c r="B27" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="C27" s="43" t="inlineStr">
+        <is>
+          <t>DFM-023.C1</t>
+        </is>
+      </c>
+      <c r="D27" s="44" t="inlineStr">
+        <is>
+          <t>Termination resistor R7 or R8 short (FMEDA SG-009 FMD-036); pass-through is not affected (R7/R8 are on the NO side)</t>
+        </is>
+      </c>
+      <c r="E27" s="44" t="inlineStr">
+        <is>
+          <t>None: the device checks only car-side messages for timeouts, so a silent camera bus is not flagged</t>
+        </is>
+      </c>
+      <c r="F27" s="44" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G27" s="44" t="inlineStr">
+        <is>
+          <t>Unchanged: stock PCS messages are lost while in intercept</t>
+        </is>
+      </c>
+      <c r="H27" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="I27" s="45" t="n">
+        <v>3</v>
+      </c>
+      <c r="J27" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="K27" s="47" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="L27" s="44" t="inlineStr"/>
+      <c r="M27" s="43" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N27" s="44" t="inlineStr">
+        <is>
+          <t>DFM-ACT-014 · open</t>
+        </is>
+      </c>
+      <c r="O27" s="49" t="inlineStr"/>
+      <c r="P27" s="49" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:P25"/>
+  <autoFilter ref="A2:P27"/>
   <mergeCells count="1">
     <mergeCell ref="A1:P1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="O3 O4 O5 O6 O7 O8 O9 O10 O11 O12 O13 O14 O15 O16 O17 O18 O19 O20 O21 O22 O23 O24 O25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this MSR row" type="list">
+    <dataValidation sqref="O3 O4 O5 O6 O7 O8 O9 O10 O11 O12 O13 O14 O15 O16 O17 O18 O19 O20 O21 O22 O23 O24 O25 O26 O27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this MSR row" type="list">
       <formula1>"Agree,Re-rate,Reject,Question"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10676,7 +11295,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LDFMEA — device, integrated panda, harness, vehicle interfaces · FMEA-MSR · rev 0.12 · BL-007&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LDFMEA — device, integrated panda, harness, vehicle interfaces · FMEA-MSR · rev 0.13 · BL-007&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>